<commit_message>
Revised Chapter 3 Handouts
</commit_message>
<xml_diff>
--- a/handouts/chapter_3_1_handout.xlsx
+++ b/handouts/chapter_3_1_handout.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\RussellStuff\Time series personal work\timeseries\handouts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\craigaj\Documents\GitHub\timeseries\handouts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03622020-F013-48B5-8F06-1294E4848C13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E350A99-383C-4E65-B7CE-9011FE7090A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{050B526A-FAB3-4422-A3BC-CA0FA5188BD4}"/>
+    <workbookView xWindow="1480" yWindow="1480" windowWidth="19200" windowHeight="11170" xr2:uid="{050B526A-FAB3-4422-A3BC-CA0FA5188BD4}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Lesson 3-1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,15 +36,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="21">
   <si>
     <t>Sum</t>
   </si>
   <si>
     <t>t</t>
-  </si>
-  <si>
-    <t>—</t>
   </si>
   <si>
     <r>
@@ -441,6 +438,35 @@
         <color theme="1"/>
         <rFont val="Times New Roman"/>
         <family val="1"/>
+      </rPr>
+      <t>k</t>
+    </r>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Computation of the Sample Cross-Correlation Function, </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Source Sans Pro"/>
+        <family val="2"/>
+      </rPr>
+      <t>r</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="subscript"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Source Sans Pro"/>
+        <family val="2"/>
       </rPr>
       <t>k</t>
     </r>
@@ -450,6 +476,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -459,31 +488,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF000000"/>
-      <name val="Source Sans Pro"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9.6"/>
       <color theme="1"/>
       <name val="Source Sans Pro"/>
       <family val="2"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9.6"/>
@@ -526,6 +534,27 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Source Sans Pro"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Source Sans Pro"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <vertAlign val="subscript"/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Source Sans Pro"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -542,12 +571,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.89999084444715716"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -570,40 +599,138 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -936,483 +1063,518 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCA80FE4-80D1-40E7-836A-EDFFE58E25C7}">
-  <dimension ref="A3:P18"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="8" max="8" width="0.54296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
+    <row r="1" spans="1:17" ht="39.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+      <c r="P1" s="11"/>
+      <c r="Q1" s="12"/>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="2"/>
+    <row r="2" spans="1:17" s="1" customFormat="1" ht="17.5" x14ac:dyDescent="0.45">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2"/>
+      <c r="I2" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="K2" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="N2" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q2" s="13" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="5" spans="1:16" s="3" customFormat="1" ht="17.5" x14ac:dyDescent="0.45">
-      <c r="A5" s="4" t="s">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B3" s="4">
+        <v>21</v>
+      </c>
+      <c r="C3" s="4">
+        <v>14</v>
+      </c>
+      <c r="D3" s="4">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="8">
+        <v>-1</v>
+      </c>
+      <c r="N3" s="7"/>
+      <c r="O3" s="5">
         <v>3</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="P3" s="5">
+        <v>5</v>
+      </c>
+      <c r="Q3" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>20</v>
+      </c>
+      <c r="C4" s="4">
+        <v>16</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="7"/>
+      <c r="N4" s="7"/>
+      <c r="O4" s="5">
+        <v>-5</v>
+      </c>
+      <c r="P4" s="5">
+        <v>-2</v>
+      </c>
+      <c r="Q4" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>17</v>
+      </c>
+      <c r="C5" s="4">
+        <v>18</v>
+      </c>
+      <c r="D5" s="4">
+        <v>-3</v>
+      </c>
+      <c r="E5" s="4">
+        <v>9</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="7"/>
+      <c r="J5" s="7"/>
+      <c r="K5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="7"/>
+      <c r="N5" s="7"/>
+      <c r="O5" s="5">
+        <v>-6</v>
+      </c>
+      <c r="P5" s="5">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A6" s="4">
         <v>4</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="B6" s="4">
+        <v>15</v>
+      </c>
+      <c r="C6" s="4">
+        <v>17</v>
+      </c>
+      <c r="D6" s="4">
+        <v>-5</v>
+      </c>
+      <c r="E6" s="4">
+        <v>25</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="7"/>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="7"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="5">
+        <v>2</v>
+      </c>
+      <c r="P6" s="5">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="5">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="B7" s="4">
+        <v>18</v>
+      </c>
+      <c r="C7" s="4">
+        <v>12</v>
+      </c>
+      <c r="D7" s="4">
+        <v>-2</v>
+      </c>
+      <c r="E7" s="4">
+        <v>4</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="7"/>
+      <c r="J7" s="7"/>
+      <c r="K7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="7"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="5">
+        <v>-3</v>
+      </c>
+      <c r="P7" s="5">
+        <v>-12</v>
+      </c>
+      <c r="Q7" s="5">
+        <v>-6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A8" s="4">
         <v>6</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="B8" s="4">
+        <v>21</v>
+      </c>
+      <c r="C8" s="4">
+        <v>10</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4">
+        <v>1</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="5">
+        <v>-20</v>
+      </c>
+      <c r="P8" s="5">
+        <v>-10</v>
+      </c>
+      <c r="Q8" s="5">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A9" s="4">
         <v>7</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="B9" s="4">
+        <v>21</v>
+      </c>
+      <c r="C9" s="4">
+        <v>11</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+      <c r="N9" s="7"/>
+      <c r="O9" s="5">
+        <v>-8</v>
+      </c>
+      <c r="P9" s="5">
+        <v>-4</v>
+      </c>
+      <c r="Q9" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A10" s="4">
         <v>8</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="B10" s="4">
+        <v>24</v>
+      </c>
+      <c r="C10" s="4">
+        <v>16</v>
+      </c>
+      <c r="D10" s="4">
+        <v>4</v>
+      </c>
+      <c r="E10" s="4">
+        <v>16</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="5">
+        <v>1</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q10" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A11" s="4">
         <v>9</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="B11" s="4">
+        <v>22</v>
+      </c>
+      <c r="C11" s="4">
+        <v>14</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+      <c r="N11" s="7"/>
+      <c r="O11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="P11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q11" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A12" s="4">
         <v>10</v>
       </c>
-      <c r="J5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="O5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="P5" s="6" t="s">
+      <c r="B12" s="4">
+        <v>21</v>
+      </c>
+      <c r="C12" s="4">
+        <v>22</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+      <c r="N12" s="7"/>
+      <c r="O12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="P12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q12" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="4">
+        <v>200</v>
+      </c>
+      <c r="C13" s="4">
+        <v>150</v>
+      </c>
+      <c r="D13" s="4">
+        <v>0</v>
+      </c>
+      <c r="E13" s="4">
+        <v>62</v>
+      </c>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="5">
+        <v>-36</v>
+      </c>
+      <c r="P13" s="5">
+        <v>-18</v>
+      </c>
+      <c r="Q13" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="17" x14ac:dyDescent="0.35">
+      <c r="D14" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="E14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
+      <c r="N14" s="7"/>
+      <c r="O14" s="5">
+        <v>-3.6</v>
+      </c>
+      <c r="P14" s="5">
+        <v>-1.8</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>0.3</v>
+      </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="7">
-        <v>1</v>
-      </c>
-      <c r="B6" s="7">
-        <v>21</v>
-      </c>
-      <c r="C6" s="7">
-        <v>14</v>
-      </c>
-      <c r="D6" s="7">
-        <v>1</v>
-      </c>
-      <c r="E6" s="7">
-        <v>1</v>
-      </c>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="8">
-        <v>-1</v>
-      </c>
-      <c r="M6" s="10"/>
-      <c r="N6" s="8">
-        <v>3</v>
-      </c>
-      <c r="O6" s="8">
-        <v>5</v>
-      </c>
-      <c r="P6" s="8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7" s="7">
-        <v>2</v>
-      </c>
-      <c r="B7" s="7">
-        <v>20</v>
-      </c>
-      <c r="C7" s="7">
-        <v>16</v>
-      </c>
-      <c r="D7" s="7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="10"/>
-      <c r="M7" s="10"/>
-      <c r="N7" s="8">
-        <v>-5</v>
-      </c>
-      <c r="O7" s="8">
-        <v>-2</v>
-      </c>
-      <c r="P7" s="8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8" s="7">
-        <v>3</v>
-      </c>
-      <c r="B8" s="7">
-        <v>17</v>
-      </c>
-      <c r="C8" s="7">
+    <row r="15" spans="1:17" ht="17" x14ac:dyDescent="0.35">
+      <c r="D15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7">
-        <v>-3</v>
-      </c>
-      <c r="E8" s="7">
-        <v>9</v>
-      </c>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
-      <c r="M8" s="10"/>
-      <c r="N8" s="8">
-        <v>-6</v>
-      </c>
-      <c r="O8" s="8">
-        <v>3</v>
-      </c>
-      <c r="P8" s="8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" s="7">
-        <v>4</v>
-      </c>
-      <c r="B9" s="7">
-        <v>15</v>
-      </c>
-      <c r="C9" s="7">
-        <v>17</v>
-      </c>
-      <c r="D9" s="7">
-        <v>-5</v>
-      </c>
-      <c r="E9" s="7">
-        <v>25</v>
-      </c>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="8">
-        <v>2</v>
-      </c>
-      <c r="O9" s="8">
-        <v>2</v>
-      </c>
-      <c r="P9" s="8">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A10" s="7">
-        <v>5</v>
-      </c>
-      <c r="B10" s="7">
-        <v>18</v>
-      </c>
-      <c r="C10" s="7">
-        <v>12</v>
-      </c>
-      <c r="D10" s="7">
-        <v>-2</v>
-      </c>
-      <c r="E10" s="7">
-        <v>4</v>
-      </c>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="8">
-        <v>-3</v>
-      </c>
-      <c r="O10" s="8">
-        <v>-12</v>
-      </c>
-      <c r="P10" s="8">
-        <v>-6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A11" s="7">
-        <v>6</v>
-      </c>
-      <c r="B11" s="7">
-        <v>21</v>
-      </c>
-      <c r="C11" s="7">
-        <v>10</v>
-      </c>
-      <c r="D11" s="7">
-        <v>1</v>
-      </c>
-      <c r="E11" s="7">
-        <v>1</v>
-      </c>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="8">
-        <v>-20</v>
-      </c>
-      <c r="O11" s="8">
-        <v>-10</v>
-      </c>
-      <c r="P11" s="8">
-        <v>-5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A12" s="7">
-        <v>7</v>
-      </c>
-      <c r="B12" s="7">
-        <v>21</v>
-      </c>
-      <c r="C12" s="7">
-        <v>11</v>
-      </c>
-      <c r="D12" s="7">
-        <v>1</v>
-      </c>
-      <c r="E12" s="7">
-        <v>1</v>
-      </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
-      <c r="N12" s="8">
-        <v>-8</v>
-      </c>
-      <c r="O12" s="8">
-        <v>-4</v>
-      </c>
-      <c r="P12" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13" s="7">
-        <v>8</v>
-      </c>
-      <c r="B13" s="7">
-        <v>24</v>
-      </c>
-      <c r="C13" s="7">
-        <v>16</v>
-      </c>
-      <c r="D13" s="7">
-        <v>4</v>
-      </c>
-      <c r="E13" s="7">
-        <v>16</v>
-      </c>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
-      <c r="N13" s="8">
-        <v>1</v>
-      </c>
-      <c r="O13" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="P13" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A14" s="7">
-        <v>9</v>
-      </c>
-      <c r="B14" s="7">
-        <v>22</v>
-      </c>
-      <c r="C14" s="7">
-        <v>14</v>
-      </c>
-      <c r="D14" s="7">
-        <v>2</v>
-      </c>
-      <c r="E14" s="7">
-        <v>4</v>
-      </c>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="O14" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="P14" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A15" s="7">
-        <v>10</v>
-      </c>
-      <c r="B15" s="7">
-        <v>21</v>
-      </c>
-      <c r="C15" s="7">
-        <v>22</v>
-      </c>
-      <c r="D15" s="7">
-        <v>1</v>
-      </c>
-      <c r="E15" s="7">
-        <v>1</v>
-      </c>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="P15" s="10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A16" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="B16" s="7">
-        <v>200</v>
-      </c>
-      <c r="C16" s="7">
-        <v>150</v>
-      </c>
-      <c r="D16" s="7">
-        <v>0</v>
-      </c>
-      <c r="E16" s="7">
-        <v>62</v>
-      </c>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="10"/>
-      <c r="M16" s="10"/>
-      <c r="N16" s="8">
-        <v>-36</v>
-      </c>
-      <c r="O16" s="8">
-        <v>-18</v>
-      </c>
-      <c r="P16" s="8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="7:16" ht="17" x14ac:dyDescent="0.35">
-      <c r="G17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="10"/>
-      <c r="M17" s="10"/>
-      <c r="N17" s="8">
-        <v>-3.6</v>
-      </c>
-      <c r="O17" s="8">
-        <v>-1.8</v>
-      </c>
-      <c r="P17" s="8">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="18" spans="7:16" ht="17" x14ac:dyDescent="0.35">
-      <c r="G18" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="10"/>
-      <c r="M18" s="10"/>
-      <c r="N18" s="8">
+      <c r="I15" s="14"/>
+      <c r="J15" s="14"/>
+      <c r="K15" s="14"/>
+      <c r="L15" s="14"/>
+      <c r="M15" s="14"/>
+      <c r="N15" s="14"/>
+      <c r="O15" s="15">
         <v>-0.42399999999999999</v>
       </c>
-      <c r="O18" s="8">
+      <c r="P15" s="15">
         <v>-0.21199999999999999</v>
       </c>
-      <c r="P18" s="8">
+      <c r="Q15" s="15">
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:Q1"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>